<commit_message>
only write one variable to stata output
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/test_stata_output.xlsx
+++ b/tests/testthat/excel/test_stata_output.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" state="visible" r:id="rId2"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="37">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -239,7 +239,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -339,7 +339,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I28"/>
-  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -684,7 +684,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -701,12 +701,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A3"/>
-  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A3:C3"/>
+  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>36</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>